<commit_message>
Actualizar productos.xlsx e imagenes
</commit_message>
<xml_diff>
--- a/tienda/productos.xlsx
+++ b/tienda/productos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9af133bd758b7a26/Documentos/novacenter/tienda/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C056F41-D6D9-4CA5-82C2-3CDFE1A3B964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E9E61A4-74B9-4B31-B43C-90CCC9F8128C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1AD9C8EF-0A24-44F4-88D7-7B3BBBFBD485}"/>
+    <workbookView xWindow="7200" yWindow="30" windowWidth="21600" windowHeight="11385" xr2:uid="{A4B675B1-F77A-4BEE-9EF9-5ECEC5AAEFBD}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -4984,7 +4984,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA06D5F8-F8BA-4DE0-87C4-C81D57BB73BF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B70F4FB-D88C-4329-A0F7-5D0EE33304B4}">
   <dimension ref="A1:N839"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -5272,7 +5272,7 @@
         <v>297</v>
       </c>
       <c r="L7">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M7">
         <v>0</v>
@@ -5644,7 +5644,7 @@
         <v>1700</v>
       </c>
       <c r="L16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M16">
         <v>0</v>
@@ -7605,7 +7605,7 @@
         <v>3505</v>
       </c>
       <c r="L62">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M62">
         <v>0</v>
@@ -9246,7 +9246,7 @@
         <v>12000</v>
       </c>
       <c r="L101">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M101">
         <v>0</v>
@@ -9636,7 +9636,7 @@
         <v>18000</v>
       </c>
       <c r="L110">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M110">
         <v>0</v>
@@ -10668,7 +10668,7 @@
         <v>8550</v>
       </c>
       <c r="K134">
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="L134">
         <v>2</v>
@@ -11843,7 +11843,7 @@
         <v>1230</v>
       </c>
       <c r="L162">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M162">
         <v>0</v>
@@ -13132,7 +13132,7 @@
         <v>2000</v>
       </c>
       <c r="L193">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M193">
         <v>0</v>
@@ -14401,7 +14401,7 @@
         <v>1365</v>
       </c>
       <c r="L223">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="M223">
         <v>0</v>
@@ -14577,7 +14577,7 @@
         <v>1929</v>
       </c>
       <c r="L227">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M227">
         <v>0</v>
@@ -14753,7 +14753,7 @@
         <v>5418</v>
       </c>
       <c r="L231">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M231">
         <v>0</v>
@@ -16093,7 +16093,7 @@
         <v>0</v>
       </c>
       <c r="L262">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M262">
         <v>0</v>
@@ -17763,7 +17763,7 @@
         <v>3225.8</v>
       </c>
       <c r="L302">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="M302">
         <v>0</v>
@@ -18015,7 +18015,7 @@
         <v>3000</v>
       </c>
       <c r="L308">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M308">
         <v>0</v>
@@ -19040,7 +19040,7 @@
         <v>1250</v>
       </c>
       <c r="L333">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="M333">
         <v>0</v>
@@ -22544,7 +22544,7 @@
         <v>20000</v>
       </c>
       <c r="L417">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M417">
         <v>0</v>
@@ -22676,7 +22676,7 @@
         <v>20000</v>
       </c>
       <c r="L420">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="M420">
         <v>0</v>
@@ -22764,7 +22764,7 @@
         <v>20000</v>
       </c>
       <c r="L422">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="M422">
         <v>0</v>
@@ -22808,7 +22808,7 @@
         <v>26000</v>
       </c>
       <c r="L423">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M423">
         <v>0</v>
@@ -22852,7 +22852,7 @@
         <v>20000</v>
       </c>
       <c r="L424">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M424">
         <v>0</v>
@@ -22940,7 +22940,7 @@
         <v>22000</v>
       </c>
       <c r="L426">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M426">
         <v>0</v>
@@ -23186,7 +23186,7 @@
         <v>22400</v>
       </c>
       <c r="L432">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M432">
         <v>0</v>
@@ -23356,7 +23356,7 @@
         <v>23000</v>
       </c>
       <c r="L436">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M436">
         <v>0</v>
@@ -23485,7 +23485,7 @@
         <v>20000</v>
       </c>
       <c r="L439">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M439">
         <v>0</v>
@@ -23573,7 +23573,7 @@
         <v>22000</v>
       </c>
       <c r="L441">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="M441">
         <v>0</v>
@@ -23599,25 +23599,25 @@
         <v>820</v>
       </c>
       <c r="F442">
-        <v>13050</v>
+        <v>14490</v>
       </c>
       <c r="G442">
-        <v>45000</v>
+        <v>50000</v>
       </c>
       <c r="H442">
         <v>21</v>
       </c>
       <c r="I442">
-        <v>13050</v>
+        <v>14490</v>
       </c>
       <c r="J442">
-        <v>22567.4</v>
+        <v>14490</v>
       </c>
       <c r="K442">
-        <v>25000</v>
+        <v>24000</v>
       </c>
       <c r="L442">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M442">
         <v>0</v>
@@ -23643,25 +23643,25 @@
         <v>197</v>
       </c>
       <c r="F443">
-        <v>12750</v>
+        <v>11710</v>
       </c>
       <c r="G443">
-        <v>45000</v>
+        <v>40000</v>
       </c>
       <c r="H443">
         <v>21</v>
       </c>
       <c r="I443">
-        <v>12750</v>
+        <v>11710</v>
       </c>
       <c r="J443">
-        <v>24106.400000000001</v>
+        <v>11710</v>
       </c>
       <c r="K443">
-        <v>22000</v>
+        <v>20000</v>
       </c>
       <c r="L443">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M443">
         <v>0</v>
@@ -23690,7 +23690,7 @@
         <v>15860</v>
       </c>
       <c r="G444">
-        <v>48000</v>
+        <v>58000</v>
       </c>
       <c r="H444">
         <v>21</v>
@@ -23746,7 +23746,7 @@
         <v>24000</v>
       </c>
       <c r="L445">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M445">
         <v>0</v>
@@ -23790,7 +23790,7 @@
         <v>21000</v>
       </c>
       <c r="L446">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M446">
         <v>0</v>
@@ -23916,7 +23916,7 @@
         <v>30000</v>
       </c>
       <c r="L449">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M449">
         <v>0</v>
@@ -23957,7 +23957,7 @@
         <v>25000</v>
       </c>
       <c r="L450">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M450">
         <v>0</v>
@@ -24358,25 +24358,25 @@
         <v>28</v>
       </c>
       <c r="F460">
-        <v>11381</v>
+        <v>13175</v>
       </c>
       <c r="G460">
-        <v>40000</v>
+        <v>46304.9</v>
       </c>
       <c r="H460">
         <v>21</v>
       </c>
       <c r="I460">
-        <v>11381</v>
+        <v>13175</v>
       </c>
       <c r="J460">
-        <v>11381</v>
+        <v>13175</v>
       </c>
       <c r="K460">
-        <v>20000</v>
+        <v>22000</v>
       </c>
       <c r="L460">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M460">
         <v>0</v>
@@ -25059,7 +25059,7 @@
         <v>20000</v>
       </c>
       <c r="L476">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M476">
         <v>0</v>
@@ -25100,7 +25100,7 @@
         <v>20000</v>
       </c>
       <c r="L477">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M477">
         <v>0</v>
@@ -25141,7 +25141,7 @@
         <v>20000</v>
       </c>
       <c r="L478">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M478">
         <v>0</v>
@@ -25229,7 +25229,7 @@
         <v>18000</v>
       </c>
       <c r="L480">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="M480">
         <v>0</v>
@@ -25317,7 +25317,7 @@
         <v>21000</v>
       </c>
       <c r="L482">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M482">
         <v>0</v>
@@ -25402,7 +25402,7 @@
         <v>20000</v>
       </c>
       <c r="L484">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="M484">
         <v>0</v>
@@ -25575,7 +25575,7 @@
         <v>22000</v>
       </c>
       <c r="L488">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M488">
         <v>0</v>
@@ -25663,7 +25663,7 @@
         <v>23000</v>
       </c>
       <c r="L490">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="M490">
         <v>0</v>
@@ -25707,7 +25707,7 @@
         <v>24000</v>
       </c>
       <c r="L491">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M491">
         <v>0</v>
@@ -25821,7 +25821,7 @@
         <v>173</v>
       </c>
       <c r="F494">
-        <v>8897</v>
+        <v>10000</v>
       </c>
       <c r="G494">
         <v>40000</v>
@@ -25830,16 +25830,16 @@
         <v>21</v>
       </c>
       <c r="I494">
-        <v>8897</v>
+        <v>10000</v>
       </c>
       <c r="J494">
-        <v>18164.099999999999</v>
+        <v>10000</v>
       </c>
       <c r="K494">
         <v>20000</v>
       </c>
       <c r="L494">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="M494">
         <v>0</v>
@@ -25868,7 +25868,7 @@
         <v>12408</v>
       </c>
       <c r="G495">
-        <v>42000</v>
+        <v>45000</v>
       </c>
       <c r="H495">
         <v>21</v>
@@ -25956,7 +25956,7 @@
         <v>11374</v>
       </c>
       <c r="G497">
-        <v>42000</v>
+        <v>45000</v>
       </c>
       <c r="H497">
         <v>21</v>
@@ -26015,7 +26015,7 @@
         <v>20000</v>
       </c>
       <c r="L498">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M498">
         <v>0</v>
@@ -26100,7 +26100,7 @@
         <v>20000</v>
       </c>
       <c r="L500">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M500">
         <v>0</v>
@@ -26226,7 +26226,7 @@
         <v>24000</v>
       </c>
       <c r="L503">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M503">
         <v>0</v>
@@ -26255,7 +26255,7 @@
         <v>17400</v>
       </c>
       <c r="G504">
-        <v>65000</v>
+        <v>60000</v>
       </c>
       <c r="H504">
         <v>21</v>
@@ -26270,7 +26270,7 @@
         <v>29000</v>
       </c>
       <c r="L504">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M504">
         <v>0</v>
@@ -26299,7 +26299,7 @@
         <v>19860</v>
       </c>
       <c r="G505">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="H505">
         <v>21</v>
@@ -26704,7 +26704,7 @@
         <v>22000</v>
       </c>
       <c r="L514">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M514">
         <v>0</v>
@@ -26833,7 +26833,7 @@
         <v>21500</v>
       </c>
       <c r="L517">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M517">
         <v>0</v>
@@ -27006,7 +27006,7 @@
         <v>30000</v>
       </c>
       <c r="L521">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M521">
         <v>0</v>
@@ -27079,7 +27079,7 @@
         <v>17574</v>
       </c>
       <c r="G523">
-        <v>60000</v>
+        <v>55000</v>
       </c>
       <c r="H523">
         <v>21</v>
@@ -27094,7 +27094,7 @@
         <v>30000</v>
       </c>
       <c r="L523">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M523">
         <v>0</v>
@@ -27182,7 +27182,7 @@
         <v>55000</v>
       </c>
       <c r="L525">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M525">
         <v>0</v>
@@ -27712,7 +27712,7 @@
         <v>931</v>
       </c>
       <c r="F538">
-        <v>8496</v>
+        <v>8183</v>
       </c>
       <c r="G538">
         <v>40000</v>
@@ -27721,16 +27721,16 @@
         <v>21</v>
       </c>
       <c r="I538">
-        <v>8496</v>
+        <v>8183</v>
       </c>
       <c r="J538">
-        <v>17221.400000000001</v>
+        <v>16586.900000000001</v>
       </c>
       <c r="K538">
-        <v>20000</v>
+        <v>18000</v>
       </c>
       <c r="L538">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="M538">
         <v>0</v>
@@ -27994,7 +27994,7 @@
         <v>23000</v>
       </c>
       <c r="L544">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M544">
         <v>0</v>
@@ -28020,25 +28020,25 @@
         <v>1021</v>
       </c>
       <c r="F545">
-        <v>15700</v>
+        <v>16500</v>
       </c>
       <c r="G545">
-        <v>52000</v>
+        <v>55000</v>
       </c>
       <c r="H545">
         <v>21</v>
       </c>
       <c r="I545">
-        <v>15700</v>
+        <v>16500</v>
       </c>
       <c r="J545">
-        <v>28125</v>
+        <v>29558.1</v>
       </c>
       <c r="K545">
-        <v>28125</v>
+        <v>26000</v>
       </c>
       <c r="L545">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M545">
         <v>0</v>
@@ -28082,7 +28082,7 @@
         <v>25000</v>
       </c>
       <c r="L546">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M546">
         <v>0</v>
@@ -28258,7 +28258,7 @@
         <v>24000</v>
       </c>
       <c r="L550">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M550">
         <v>0</v>
@@ -28560,7 +28560,7 @@
         <v>25000</v>
       </c>
       <c r="L557">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M557">
         <v>0</v>
@@ -28604,7 +28604,7 @@
         <v>23000</v>
       </c>
       <c r="L558">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M558">
         <v>0</v>
@@ -30568,7 +30568,7 @@
         <v>233</v>
       </c>
       <c r="L604">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M604">
         <v>0</v>
@@ -30612,7 +30612,7 @@
         <v>9000</v>
       </c>
       <c r="L605">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M605">
         <v>0</v>
@@ -30653,7 +30653,7 @@
         <v>8000</v>
       </c>
       <c r="L606">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="M606">
         <v>0</v>
@@ -31254,7 +31254,7 @@
         <v>527</v>
       </c>
       <c r="L620">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M620">
         <v>0</v>
@@ -32716,7 +32716,7 @@
         <v>8000</v>
       </c>
       <c r="L655">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M655">
         <v>0</v>
@@ -32804,7 +32804,7 @@
         <v>10000</v>
       </c>
       <c r="L657">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M657">
         <v>0</v>
@@ -36551,7 +36551,7 @@
         <v>9493</v>
       </c>
       <c r="L744">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M744">
         <v>0</v>
@@ -40102,7 +40102,7 @@
         <v>12730</v>
       </c>
       <c r="L829">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M829">
         <v>0</v>
@@ -40395,7 +40395,7 @@
         <v>3613.6</v>
       </c>
       <c r="L836">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M836">
         <v>0</v>

</xml_diff>